<commit_message>
feat(bar-business-plan): entregables EN regenerados tras la revisión final (mismas cifras del caso)
aplicar_en --idempotencia + ensamblar_docx en el VPS con los arreglos de texto de 5be311da: gates G1-G9 TODO VERDE,
--autotest 20/20 y 8/8, 0 fallos de pycel, 0 diferencias, barrido sin cifras ES ni español ni no latinos. Los 100
tokens de cifras_caso.json idénticos a los de antes; 5 tokens derivados nuevos. F2-NOTAS §9.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KriAdpMP6uaswtiVvqtBvP
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bar-business-plan/bar-financial-projections.xlsx
+++ b/astro-site/public/dl/bar-business-plan/bar-financial-projections.xlsx
@@ -1293,7 +1293,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Build-out, installations, ventilation and decor of a bar with a commercial kitchen. Straight-line depreciation for the books; tax depreciation (MACRS, Section 179) can differ, so ask your CPA</t>
+          <t>Build-out, installations, ventilation and decor of a bar with a commercial kitchen, including the draft beer system. Straight-line depreciation for the books; tax depreciation (MACRS, Section 179) can differ, so ask your CPA</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Griddle, fryer, oven, refrigeration, draft beer system and bar furniture. Straight-line depreciation over the useful life you enter; tax depreciation (MACRS, Section 179) can differ, so confirm it with your CPA</t>
+          <t>Griddle, fryer, oven, refrigeration, the bar build and furniture. Straight-line depreciation over the useful life you enter; tax depreciation (MACRS, Section 179) can differ, so confirm it with your CPA</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TOTAL capacity of the space: dining room seats, bar stools and patio. Count it on your floor plan rather than copying the example: if your patio is large, capacity rises and the implied seat turns fall. Daily covers ÷ seats gives the implied seat turns in the row below</t>
+          <t>TOTAL capacity of the space: dining room seats and bar stools; add patio seats only if they are open most of the year. Count it on your floor plan rather than copying the example: counting a year-round patio raises capacity and lowers the implied seat turns. Daily covers ÷ seats gives the implied seat turns in the row below</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>You pay for the space from the day you sign. These months are a startup cost: they do NOT overlap the P&amp;L, which starts on opening day</t>
+          <t>You pay for the space from the day you sign. These months are a startup cost: they do NOT overlap the P&amp;L, which starts on opening day. If your liquor license is likely to take longer than the build-out (often 3-12 months from signing), enter the months until it is issued, or negotiate a license contingency and rent abatement in the lease.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Same example rate as the rest of on-site sales (8%: state + local). Some states add a tax on drinks served on premises; e.g. Texas: 8.25% mixed beverage sales tax (paid by the customer) + 6.7% gross receipts tax (paid by the bar): put the first here and add the second to your beverage cost %. The workbook applies this rate only to the ALCOHOLIC part of beverage sales</t>
+          <t>Same example rate as the rest of on-site sales (8%: state + local). Some states add a tax on drinks served on premises; e.g. Texas: 8.25% mixed beverage sales tax (paid by the customer) + 6.7% gross receipts tax (paid by the bar): put the first here and add 6.7% × your alcohol share (about 6 points at 90%) to your beverage cost %. The workbook applies this rate only to the ALCOHOLIC part of beverage sales</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="D8" s="29" t="inlineStr">
         <is>
-          <t>Beer &amp; wine licenses start around $3,000; full liquor runs $12,000-$400,000. In quota states you buy an existing license at market price, which costs far more; this row is an example for a state WITHOUT a quota. A license bought from another owner is an intangible asset: ask your CPA. Apply right after signing the lease: it often takes 3-12 months</t>
+          <t>Beer &amp; wine licenses start around $3,000; full liquor runs $12,000-$400,000. In quota states you buy an existing license at market price, which costs far more; this row is an example for a state WITHOUT a quota. A license bought from another owner is an intangible asset: ask your CPA. Apply right after signing the lease: it often takes 3-12 months. Most states also charge an annual or biennial renewal fee: add it to your fixed costs</t>
         </is>
       </c>
       <c r="E8" s="32" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="E24" s="34" t="inlineStr">
         <is>
-          <t>Covers each full-time employee in the "5. Staffing" tab would have to serve. In the optimistic scenario it tells you whether you need to hire</t>
+          <t>Covers each full-time employee in the "Staffing" tab would have to serve. In the optimistic scenario it tells you whether you need to hire</t>
         </is>
       </c>
     </row>
@@ -5904,10 +5904,10 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="284.25" customHeight="1">
+    <row r="29" ht="194.5" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>The gross pay, employer payroll taxes, monthly cost and annual cost columns are TOTALS for the row: for a position with two people they include both. FTE is the share of a full-time week for each person, and it is used to compare pay with the legal minimum in proportion; the TOTAL row multiplies it by the people in each position, so it gives the full-time equivalents of the whole team. The payroll tax rate and the number of pay periods are in the "0. Assumptions" tab. Tips are not modeled: bartenders, barbacks and servers are budgeted at a base wage of at least $15/h. Federal rules allow a $2.13/h cash wage with a tip credit of up to $5.12 where the state permits it; CA, OR, WA, AK, MN, MT and NV do not (DOL)</t>
+          <t>The gross pay, employer payroll taxes, monthly cost and annual cost columns are TOTALS for the row: for a position with two people they include both. The payroll tax rate and the number of pay periods are in the "0. Assumptions" tab. Tips are not modeled: bartenders, barbacks and servers are budgeted at a base wage of at least $15/h. Federal rules allow a $2.13/h cash wage with a tip credit of up to $5.12 where the state permits it; CA, OR, WA, AK, MN, MT and NV do not (DOL)</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6734,7 @@
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
         <is>
-          <t>US INDUSTRY BENCHMARKS</t>
+          <t>US INDUSTRY BENCHMARKS (sourced) AND KIT ESTIMATES</t>
         </is>
       </c>
     </row>
@@ -6782,7 +6782,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="30" customHeight="1">
+    <row r="55" ht="45" customHeight="1">
       <c r="A55" t="inlineStr">
         <is>
           <t>Pour cost, whole bar</t>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="D55" s="17" t="inlineStr">
         <is>
-          <t>The beverage cost in this example (the "Beverage cost" row of "0. Assumptions") includes garnish and spillage</t>
+          <t>The beverage cost in this example (the "Cost of goods sold on BEVERAGE sales" row of "0. Assumptions") includes garnish and spillage</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="D69" s="17" t="inlineStr">
         <is>
-          <t>Enter your state's floor on "0. Assumptions"; there is no union agreement table to copy</t>
+          <t>Enter your state's floor on "0. Assumptions"; check your state and city rates at dol.gov</t>
         </is>
       </c>
     </row>

</xml_diff>